<commit_message>
figuring out what fDOM is doing
</commit_message>
<xml_diff>
--- a/correlations/multiple_regressions/regression_paper_final.xlsx
+++ b/correlations/multiple_regressions/regression_paper_final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\correlations\multiple_regressions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\correlations\multiple_regressions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42240731-2242-4D3A-9CDF-8E0F4B0FC088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EA8053-F32F-4FA9-BE0A-0311497B702B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45D0A2E9-A66C-4C74-B9CB-F5D4797C5B3E}"/>
+    <workbookView xWindow="23064" yWindow="624" windowWidth="21600" windowHeight="11292" xr2:uid="{45D0A2E9-A66C-4C74-B9CB-F5D4797C5B3E}"/>
   </bookViews>
   <sheets>
     <sheet name="tauc correlations (no st7)" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="77">
   <si>
     <t xml:space="preserve">Aich Hysteresis </t>
   </si>
@@ -268,6 +268,9 @@
   <si>
     <t xml:space="preserve">Summer Up, Spring Down </t>
   </si>
+  <si>
+    <t>fDOM</t>
+  </si>
 </sst>
 </file>
 
@@ -277,7 +280,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -314,6 +317,14 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -377,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -422,6 +433,24 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3937,7 +3966,7 @@
                   <c:v>8.9326261366187695E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6283799610675601E-2</c:v>
+                  <c:v>0.146283799610675</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.11077055296162799</c:v>
@@ -7658,7 +7687,7 @@
                   <c:v>8.9326261366187695E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6283799610675601E-2</c:v>
+                  <c:v>0.146283799610675</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.11077055296162799</c:v>
@@ -10340,7 +10369,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'tauc correlations (no st7)'!$BQ$2:$BQ$9</c:f>
+              <c:f>'tauc correlations (no st7)'!$BR$2:$BR$9</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="8"/>
@@ -10498,7 +10527,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'tauc correlations (no st7)'!$BE$2:$BE$9</c:f>
+              <c:f>'tauc correlations (no st7)'!$BF$2:$BF$9</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="8"/>
@@ -12631,7 +12660,7 @@
                   <c:v>8.9326261366187695E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6283799610675601E-2</c:v>
+                  <c:v>0.146283799610675</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.11077055296162799</c:v>
@@ -14781,7 +14810,7 @@
                   <c:v>8.9326261366187695E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6283799610675601E-2</c:v>
+                  <c:v>0.146283799610675</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.11077055296162799</c:v>
@@ -18496,7 +18525,7 @@
                   <c:v>8.9326261366187695E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6283799610675601E-2</c:v>
+                  <c:v>0.146283799610675</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.11077055296162799</c:v>
@@ -35273,7 +35302,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78D79D4C-F839-48FE-8429-4CA22E52E7DC}">
-  <dimension ref="A1:BQ74"/>
+  <dimension ref="A1:BR74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" customWidth="1"/>
@@ -35288,9 +35317,10 @@
     <col min="55" max="55" width="10.7109375" customWidth="1"/>
     <col min="56" max="58" width="11.5703125" customWidth="1"/>
     <col min="60" max="60" width="13.85546875" customWidth="1"/>
+    <col min="62" max="62" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" ht="48" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:70" ht="48" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -35346,63 +35376,68 @@
       <c r="AW1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="AX1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="AY1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="BE1" s="4" t="s">
+      <c r="BF1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="BF1" s="4"/>
       <c r="BH1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="BI1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BJ1" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="BK1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BP1" s="3" t="s">
+      <c r="BQ1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BR1" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
@@ -35463,65 +35498,70 @@
       <c r="AW2" s="6">
         <v>0.17369777575697301</v>
       </c>
-      <c r="AX2" s="8">
+      <c r="AX2" s="7">
+        <v>1.7836570943256701E-2</v>
+      </c>
+      <c r="AY2" s="8">
         <v>1.1737788669959504</v>
       </c>
-      <c r="AY2" s="8">
+      <c r="AZ2" s="8">
         <v>-1.5</v>
       </c>
-      <c r="AZ2" s="8">
+      <c r="BA2" s="8">
         <v>1.25</v>
       </c>
-      <c r="BA2" s="8">
+      <c r="BB2" s="8">
         <v>2.75</v>
       </c>
-      <c r="BB2" s="10">
-        <f>AZ2/BD2</f>
+      <c r="BC2" s="10">
+        <f>BA2/BE2</f>
         <v>0.3125</v>
       </c>
-      <c r="BC2" s="10">
-        <f>BA2/BD2</f>
+      <c r="BD2" s="10">
+        <f>BB2/BE2</f>
         <v>0.6875</v>
       </c>
-      <c r="BD2" s="8">
+      <c r="BE2" s="8">
         <v>4</v>
       </c>
-      <c r="BE2" s="10">
+      <c r="BF2" s="10">
         <v>0.30708458237534503</v>
       </c>
-      <c r="BF2" s="8"/>
       <c r="BH2" s="5" t="s">
         <v>17</v>
       </c>
       <c r="BI2" s="6">
         <v>0.13984116014494999</v>
       </c>
-      <c r="BJ2" s="8">
+      <c r="BJ2">
+        <v>-0.61127875482433702</v>
+      </c>
+      <c r="BK2" s="8">
         <v>1.1737788669959504</v>
       </c>
-      <c r="BK2" s="8">
+      <c r="BL2" s="8">
         <v>-1.5</v>
       </c>
-      <c r="BL2" s="8">
+      <c r="BM2" s="8">
         <v>1.25</v>
       </c>
-      <c r="BM2" s="8">
+      <c r="BN2" s="8">
         <v>2.75</v>
       </c>
-      <c r="BN2" s="10">
+      <c r="BO2" s="10">
         <v>0.3125</v>
       </c>
-      <c r="BO2" s="10">
+      <c r="BP2" s="10">
         <v>0.6875</v>
       </c>
-      <c r="BP2" s="8">
+      <c r="BQ2" s="8">
         <v>4</v>
       </c>
-      <c r="BQ2" s="10">
+      <c r="BR2" s="10">
         <v>0.30708458237534503</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
@@ -35582,65 +35622,70 @@
       <c r="AW3" s="6">
         <v>9.9143945152060597E-2</v>
       </c>
-      <c r="AX3" s="8">
+      <c r="AX3" s="7">
+        <v>-0.54160608613664096</v>
+      </c>
+      <c r="AY3" s="8">
         <v>1.0182769682576838</v>
       </c>
-      <c r="AY3" s="8">
+      <c r="AZ3" s="8">
         <v>-0.63852552807902296</v>
       </c>
-      <c r="AZ3" s="8">
+      <c r="BA3" s="8">
         <v>0.25</v>
       </c>
-      <c r="BA3" s="8">
+      <c r="BB3" s="8">
         <v>0.88852552807902296</v>
       </c>
-      <c r="BB3" s="10">
-        <f>AZ3/BD3</f>
+      <c r="BC3" s="10">
+        <f>BA3/BE3</f>
         <v>0.2195822525137518</v>
       </c>
-      <c r="BC3" s="10">
-        <f>BA3/BD3</f>
+      <c r="BD3" s="10">
+        <f>BB3/BE3</f>
         <v>0.7804177474862507</v>
       </c>
-      <c r="BD3" s="8">
+      <c r="BE3" s="8">
         <v>1.1385255280790201</v>
       </c>
-      <c r="BE3" s="10">
+      <c r="BF3" s="10">
         <v>0.49664162355941199</v>
       </c>
-      <c r="BF3" s="8"/>
       <c r="BH3" s="5" t="s">
         <v>19</v>
       </c>
       <c r="BI3" s="6">
         <v>8.9326261366187695E-2</v>
       </c>
-      <c r="BJ3" s="8">
+      <c r="BJ3">
+        <v>-0.64117535564386996</v>
+      </c>
+      <c r="BK3" s="8">
         <v>1.0182769682576838</v>
       </c>
-      <c r="BK3" s="8">
+      <c r="BL3" s="8">
         <v>-0.63852552807902296</v>
       </c>
-      <c r="BL3" s="8">
+      <c r="BM3" s="8">
         <v>0.25</v>
       </c>
-      <c r="BM3" s="8">
+      <c r="BN3" s="8">
         <v>0.88852552807902296</v>
       </c>
-      <c r="BN3" s="10">
+      <c r="BO3" s="10">
         <v>0.2195822525137518</v>
       </c>
-      <c r="BO3" s="10">
+      <c r="BP3" s="10">
         <v>0.7804177474862507</v>
       </c>
-      <c r="BP3" s="8">
+      <c r="BQ3" s="8">
         <v>1.1385255280790201</v>
       </c>
-      <c r="BQ3" s="10">
+      <c r="BR3" s="10">
         <v>0.49664162355941199</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
@@ -35700,11 +35745,11 @@
       <c r="AW4" s="6">
         <v>0.21234239309632399</v>
       </c>
-      <c r="AX4" s="8">
+      <c r="AX4" s="7">
+        <v>-0.17637365181995501</v>
+      </c>
+      <c r="AY4" s="8">
         <v>1</v>
-      </c>
-      <c r="AY4" s="8">
-        <v>0</v>
       </c>
       <c r="AZ4" s="8">
         <v>0</v>
@@ -35712,16 +35757,18 @@
       <c r="BA4" s="8">
         <v>0</v>
       </c>
-      <c r="BB4" s="10">
+      <c r="BB4" s="8">
         <v>0</v>
       </c>
       <c r="BC4" s="10">
         <v>0</v>
       </c>
-      <c r="BD4" s="8">
+      <c r="BD4" s="10">
         <v>0</v>
       </c>
-      <c r="BE4" s="8"/>
+      <c r="BE4" s="8">
+        <v>0</v>
+      </c>
       <c r="BF4" s="8"/>
       <c r="BH4" s="5" t="s">
         <v>21</v>
@@ -35729,11 +35776,8 @@
       <c r="BI4" s="6">
         <v>4.6283799610675601E-2</v>
       </c>
-      <c r="BJ4" s="8">
+      <c r="BK4" s="8">
         <v>1</v>
-      </c>
-      <c r="BK4" s="8">
-        <v>0</v>
       </c>
       <c r="BL4" s="8">
         <v>0</v>
@@ -35741,18 +35785,21 @@
       <c r="BM4" s="8">
         <v>0</v>
       </c>
-      <c r="BN4" s="10">
+      <c r="BN4" s="8">
         <v>0</v>
       </c>
       <c r="BO4" s="10">
         <v>0</v>
       </c>
-      <c r="BP4" s="8">
+      <c r="BP4" s="10">
         <v>0</v>
       </c>
-      <c r="BQ4" s="8"/>
+      <c r="BQ4" s="8">
+        <v>0</v>
+      </c>
+      <c r="BR4" s="8"/>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -35812,63 +35859,65 @@
       <c r="AW5" s="6">
         <v>8.8732929175135894E-2</v>
       </c>
-      <c r="AX5" s="8">
+      <c r="AX5" s="6">
+        <v>1.20306787922476E-2</v>
+      </c>
+      <c r="AY5" s="8">
         <v>1.0119508062412015</v>
       </c>
-      <c r="AY5" s="8">
+      <c r="AZ5" s="8">
         <v>-1.9243966466520197</v>
       </c>
-      <c r="AZ5" s="8">
+      <c r="BA5" s="8">
         <v>3.1258759015031101</v>
       </c>
-      <c r="BA5" s="8">
+      <c r="BB5" s="8">
         <v>5.0502725481551298</v>
       </c>
-      <c r="BB5" s="10">
-        <f>AZ5/BD5</f>
+      <c r="BC5" s="10">
+        <f>BA5/BE5</f>
         <v>0.3823164318443566</v>
       </c>
-      <c r="BC5" s="10">
-        <f>BA5/BD5</f>
+      <c r="BD5" s="10">
+        <f>BB5/BE5</f>
         <v>0.61768356815564218</v>
       </c>
-      <c r="BD5" s="8">
+      <c r="BE5" s="8">
         <v>8.1761484496582497</v>
       </c>
-      <c r="BE5" s="10">
+      <c r="BF5" s="10">
         <v>0.19059894727801999</v>
       </c>
-      <c r="BF5" s="8"/>
       <c r="BH5" s="5" t="s">
         <v>26</v>
       </c>
       <c r="BI5" s="6">
         <v>0.11077055296162799</v>
       </c>
-      <c r="BJ5" s="8">
+      <c r="BK5" s="8">
         <v>1.0078290838208943</v>
       </c>
-      <c r="BK5" s="8">
+      <c r="BL5" s="8">
         <v>1.194091358120922</v>
       </c>
-      <c r="BL5" s="8">
+      <c r="BM5" s="8">
         <v>1.8447691432308699</v>
       </c>
-      <c r="BM5" s="8">
+      <c r="BN5" s="8">
         <v>0.650677785109948</v>
       </c>
-      <c r="BN5" s="10">
+      <c r="BO5" s="10">
         <v>0.73925400788123874</v>
       </c>
-      <c r="BO5" s="10">
+      <c r="BP5" s="10">
         <v>0.26074599211876454</v>
       </c>
-      <c r="BP5" s="8">
+      <c r="BQ5" s="8">
         <v>2.4954469283408098</v>
       </c>
-      <c r="BQ5" s="10"/>
+      <c r="BR5" s="10"/>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -35903,65 +35952,67 @@
       <c r="AW6" s="6">
         <v>0.10415722716452799</v>
       </c>
-      <c r="AX6" s="8">
+      <c r="AX6" s="6">
+        <v>2.8615745110634201E-2</v>
+      </c>
+      <c r="AY6" s="8">
         <v>1.0239451393319936</v>
       </c>
-      <c r="AY6" s="8">
+      <c r="AZ6" s="8">
         <v>-8.5529249332917008</v>
       </c>
-      <c r="AZ6" s="8">
+      <c r="BA6" s="8">
         <v>5.5209579590505999</v>
       </c>
-      <c r="BA6" s="8">
+      <c r="BB6" s="8">
         <v>14.073882892342301</v>
       </c>
-      <c r="BB6" s="10">
-        <f>AZ6/BD6</f>
+      <c r="BC6" s="10">
+        <f>BA6/BE6</f>
         <v>0.28175569278268175</v>
       </c>
-      <c r="BC6" s="10">
-        <f>BA6/BD6</f>
+      <c r="BD6" s="10">
+        <f>BB6/BE6</f>
         <v>0.71824430721731836</v>
       </c>
-      <c r="BD6" s="8">
+      <c r="BE6" s="8">
         <v>19.594840851392899</v>
       </c>
-      <c r="BE6" s="10">
+      <c r="BF6" s="10">
         <v>0.499861288181496</v>
       </c>
-      <c r="BF6" s="8"/>
       <c r="BH6" s="5" t="s">
         <v>28</v>
       </c>
       <c r="BI6" s="6">
         <v>5.5397551503622099E-2</v>
       </c>
-      <c r="BJ6" s="8">
+      <c r="BK6" s="8">
         <v>1.0239451393319936</v>
       </c>
-      <c r="BK6" s="8">
+      <c r="BL6" s="8">
         <v>-8.5529249332917008</v>
       </c>
-      <c r="BL6" s="8">
+      <c r="BM6" s="8">
         <v>5.5209579590505999</v>
       </c>
-      <c r="BM6" s="8">
+      <c r="BN6" s="8">
         <v>14.073882892342301</v>
       </c>
-      <c r="BN6" s="10">
+      <c r="BO6" s="10">
         <v>0.28175569278268175</v>
       </c>
-      <c r="BO6" s="10">
+      <c r="BP6" s="10">
         <v>0.71824430721731836</v>
       </c>
-      <c r="BP6" s="8">
+      <c r="BQ6" s="8">
         <v>19.594840851392899</v>
       </c>
-      <c r="BQ6" s="10">
+      <c r="BR6" s="10">
         <v>0.499861288181496</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -35996,65 +36047,67 @@
       <c r="AW7" s="6">
         <v>4.66251429291673E-2</v>
       </c>
-      <c r="AX7" s="8">
+      <c r="AX7" s="6">
+        <v>4.4113621235337297E-2</v>
+      </c>
+      <c r="AY7" s="8">
         <v>1.0275460447393339</v>
       </c>
-      <c r="AY7" s="8">
+      <c r="AZ7" s="8">
         <v>-6.8910153198931301</v>
       </c>
-      <c r="AZ7" s="8">
+      <c r="BA7" s="8">
         <v>5.1821136906510699</v>
       </c>
-      <c r="BA7" s="8">
+      <c r="BB7" s="8">
         <v>12.0731290105442</v>
       </c>
-      <c r="BB7" s="10">
-        <f>AZ7/BD7</f>
+      <c r="BC7" s="10">
+        <f>BA7/BE7</f>
         <v>0.30032111285760682</v>
       </c>
-      <c r="BC7" s="10">
-        <f>BA7/BD7</f>
+      <c r="BD7" s="10">
+        <f>BB7/BE7</f>
         <v>0.69967888714239146</v>
       </c>
-      <c r="BD7" s="8">
+      <c r="BE7" s="8">
         <v>17.2552427011953</v>
       </c>
-      <c r="BE7" s="10">
+      <c r="BF7" s="10">
         <v>0.40695810522245701</v>
       </c>
-      <c r="BF7" s="8"/>
       <c r="BH7" s="5" t="s">
         <v>30</v>
       </c>
       <c r="BI7" s="6">
         <v>6.9883057908481996E-2</v>
       </c>
-      <c r="BJ7" s="8">
+      <c r="BK7" s="8">
         <v>1.0275460447393339</v>
       </c>
-      <c r="BK7" s="8">
+      <c r="BL7" s="8">
         <v>-6.8910153198931301</v>
       </c>
-      <c r="BL7" s="8">
+      <c r="BM7" s="8">
         <v>5.1821136906510699</v>
       </c>
-      <c r="BM7" s="8">
+      <c r="BN7" s="8">
         <v>12.0731290105442</v>
       </c>
-      <c r="BN7" s="10">
+      <c r="BO7" s="10">
         <v>0.30032111285760682</v>
       </c>
-      <c r="BO7" s="10">
+      <c r="BP7" s="10">
         <v>0.69967888714239146</v>
       </c>
-      <c r="BP7" s="8">
+      <c r="BQ7" s="8">
         <v>17.2552427011953</v>
       </c>
-      <c r="BQ7" s="10">
+      <c r="BR7" s="10">
         <v>0.40695810522245701</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>26</v>
       </c>
@@ -36109,65 +36162,67 @@
       <c r="AW8" s="6">
         <v>9.0894558490112708E-3</v>
       </c>
-      <c r="AX8" s="8">
+      <c r="AX8" s="7">
+        <v>-8.0536265843332393E-3</v>
+      </c>
+      <c r="AY8" s="8">
         <v>1.0275826446035865</v>
       </c>
-      <c r="AY8" s="8">
+      <c r="AZ8" s="8">
         <v>-4.3261384988685592</v>
       </c>
-      <c r="AZ8" s="8">
+      <c r="BA8" s="8">
         <v>6.3491431999578403</v>
       </c>
-      <c r="BA8" s="8">
+      <c r="BB8" s="8">
         <v>10.675281698826399</v>
       </c>
-      <c r="BB8" s="10">
-        <f>AZ8/BD8</f>
+      <c r="BC8" s="10">
+        <f>BA8/BE8</f>
         <v>0.37294318238093693</v>
       </c>
-      <c r="BC8" s="10">
-        <f>BA8/BD8</f>
+      <c r="BD8" s="10">
+        <f>BB8/BE8</f>
         <v>0.62705681761906529</v>
       </c>
-      <c r="BD8" s="8">
+      <c r="BE8" s="8">
         <v>17.024424898784201</v>
       </c>
-      <c r="BE8" s="10">
+      <c r="BF8" s="10">
         <v>5.4056282725128302E-2</v>
       </c>
-      <c r="BF8" s="8"/>
       <c r="BH8" s="5" t="s">
         <v>32</v>
       </c>
       <c r="BI8" s="6">
         <v>7.8645648239850305E-2</v>
       </c>
-      <c r="BJ8" s="8">
+      <c r="BK8" s="8">
         <v>1.0275826446035865</v>
       </c>
-      <c r="BK8" s="8">
+      <c r="BL8" s="8">
         <v>-4.3261384988685592</v>
       </c>
-      <c r="BL8" s="8">
+      <c r="BM8" s="8">
         <v>6.3491431999578403</v>
       </c>
-      <c r="BM8" s="8">
+      <c r="BN8" s="8">
         <v>10.675281698826399</v>
       </c>
-      <c r="BN8" s="10">
+      <c r="BO8" s="10">
         <v>0.37294318238093693</v>
       </c>
-      <c r="BO8" s="10">
+      <c r="BP8" s="10">
         <v>0.62705681761906529</v>
       </c>
-      <c r="BP8" s="8">
+      <c r="BQ8" s="8">
         <v>17.024424898784201</v>
       </c>
-      <c r="BQ8" s="10">
+      <c r="BR8" s="10">
         <v>5.4056282725128302E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -36226,65 +36281,67 @@
       <c r="AW9" s="6">
         <v>2.0373962034653699E-2</v>
       </c>
-      <c r="AX9" s="8">
+      <c r="AX9" s="6">
+        <v>2.7450804091866201E-2</v>
+      </c>
+      <c r="AY9" s="8">
         <v>1.111235100018195</v>
       </c>
-      <c r="AY9" s="8">
+      <c r="AZ9" s="8">
         <v>-7.4420412056407592</v>
       </c>
-      <c r="AZ9" s="8">
+      <c r="BA9" s="8">
         <v>7.2579587943592401</v>
       </c>
-      <c r="BA9" s="8">
+      <c r="BB9" s="8">
         <v>14.7</v>
       </c>
-      <c r="BB9" s="10">
-        <f>AZ9/BD9</f>
+      <c r="BC9" s="10">
+        <f>BA9/BE9</f>
         <v>0.33053886576304825</v>
       </c>
-      <c r="BC9" s="10">
-        <f>BA9/BD9</f>
+      <c r="BD9" s="10">
+        <f>BB9/BE9</f>
         <v>0.66946113423695353</v>
       </c>
-      <c r="BD9" s="8">
+      <c r="BE9" s="8">
         <v>21.9579587943592</v>
       </c>
-      <c r="BE9" s="10">
+      <c r="BF9" s="10">
         <v>0.45125668170602201</v>
       </c>
-      <c r="BF9" s="8"/>
       <c r="BH9" s="5" t="s">
         <v>34</v>
       </c>
       <c r="BI9" s="6">
         <v>0.101236914763633</v>
       </c>
-      <c r="BJ9" s="8">
+      <c r="BK9" s="8">
         <v>1.111235100018195</v>
       </c>
-      <c r="BK9" s="8">
+      <c r="BL9" s="8">
         <v>-7.4420412056407592</v>
       </c>
-      <c r="BL9" s="8">
+      <c r="BM9" s="8">
         <v>7.2579587943592401</v>
       </c>
-      <c r="BM9" s="8">
+      <c r="BN9" s="8">
         <v>14.7</v>
       </c>
-      <c r="BN9" s="10">
+      <c r="BO9" s="10">
         <v>0.33053886576304825</v>
       </c>
-      <c r="BO9" s="10">
+      <c r="BP9" s="10">
         <v>0.66946113423695353</v>
       </c>
-      <c r="BP9" s="8">
+      <c r="BQ9" s="8">
         <v>21.9579587943592</v>
       </c>
-      <c r="BQ9" s="10">
+      <c r="BR9" s="10">
         <v>0.45125668170602201</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>28</v>
       </c>
@@ -36337,7 +36394,7 @@
         <v>14.7</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>30</v>
       </c>
@@ -36390,7 +36447,7 @@
         <v>12.423125365279599</v>
       </c>
     </row>
-    <row r="12" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:70" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>32</v>
       </c>
@@ -36443,7 +36500,7 @@
         <v>2.75</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
@@ -36504,7 +36561,7 @@
       </c>
       <c r="BI13" s="12"/>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>40</v>
       </c>
@@ -36569,7 +36626,7 @@
         <v>0.85582878233347637</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>43</v>
       </c>
@@ -36634,7 +36691,7 @@
         <v>0.73244290467040096</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>46</v>
       </c>
@@ -36684,7 +36741,7 @@
         <v>0.62542006653856141</v>
       </c>
     </row>
-    <row r="17" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>48</v>
       </c>
@@ -36734,7 +36791,7 @@
         <v>1.8767280512430116E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>50</v>
       </c>
@@ -36784,7 +36841,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>52</v>
       </c>
@@ -36822,7 +36879,7 @@
         <v>48.251680680319097</v>
       </c>
     </row>
-    <row r="20" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>53</v>
       </c>
@@ -36866,7 +36923,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:69" x14ac:dyDescent="0.25">
       <c r="K21" s="8"/>
       <c r="AV21" s="15"/>
       <c r="AW21" s="15" t="s">
@@ -36901,7 +36958,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>60</v>
       </c>
@@ -36944,7 +37001,7 @@
         <v>3.7028931578258539E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:68" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:69" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>0</v>
       </c>
@@ -37007,7 +37064,7 @@
         <v>3.5221081783223926E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>17</v>
       </c>
@@ -37072,7 +37129,7 @@
       <c r="BL24" s="14"/>
       <c r="BM24" s="14"/>
     </row>
-    <row r="25" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>19</v>
       </c>
@@ -37113,7 +37170,7 @@
       </c>
       <c r="M25" s="8"/>
     </row>
-    <row r="26" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>23</v>
       </c>
@@ -37204,7 +37261,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -37273,7 +37330,7 @@
         <v>-1.1548698044594019E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>40</v>
       </c>
@@ -37366,7 +37423,7 @@
         <v>0.70781745311554278</v>
       </c>
     </row>
-    <row r="29" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>43</v>
       </c>
@@ -37459,7 +37516,7 @@
         <v>8.3283463983663125E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>46</v>
       </c>
@@ -37498,7 +37555,7 @@
       </c>
       <c r="M30" s="8"/>
     </row>
-    <row r="31" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>48</v>
       </c>
@@ -37536,8 +37593,25 @@
         <v>14.7819327483883</v>
       </c>
       <c r="M31" s="8"/>
+      <c r="AU31" s="17"/>
+      <c r="AV31" t="s">
+        <v>74</v>
+      </c>
+      <c r="BE31" s="17"/>
+      <c r="BF31" s="17"/>
+      <c r="BG31" s="17"/>
+      <c r="BH31" s="17"/>
+      <c r="BI31" s="17"/>
+      <c r="BJ31" s="17"/>
+      <c r="BK31" s="17"/>
+      <c r="BL31" s="17"/>
+      <c r="BM31" s="17"/>
+      <c r="BN31" s="17"/>
+      <c r="BO31" s="17"/>
+      <c r="BP31" s="17"/>
+      <c r="BQ31" s="17"/>
     </row>
-    <row r="32" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>50</v>
       </c>
@@ -37575,8 +37649,22 @@
         <v>15.671540073004801</v>
       </c>
       <c r="M32" s="8"/>
+      <c r="AU32" s="17"/>
+      <c r="BE32" s="17"/>
+      <c r="BF32" s="17"/>
+      <c r="BG32" s="17"/>
+      <c r="BH32" s="17"/>
+      <c r="BI32" s="17"/>
+      <c r="BJ32" s="17"/>
+      <c r="BK32" s="17"/>
+      <c r="BL32" s="17"/>
+      <c r="BM32" s="17"/>
+      <c r="BN32" s="17"/>
+      <c r="BO32" s="17"/>
+      <c r="BP32" s="17"/>
+      <c r="BQ32" s="17"/>
     </row>
-    <row r="33" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>52</v>
       </c>
@@ -37614,16 +37702,26 @@
         <v>48.251680680319097</v>
       </c>
       <c r="M33" s="8"/>
-      <c r="AV33" s="12" t="s">
+      <c r="AU33" s="17"/>
+      <c r="AV33" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="AW33" s="12"/>
-      <c r="BH33" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI33" s="12"/>
+      <c r="AW33" s="24"/>
+      <c r="BE33" s="17"/>
+      <c r="BF33" s="17"/>
+      <c r="BG33" s="17"/>
+      <c r="BH33" s="19"/>
+      <c r="BI33" s="19"/>
+      <c r="BJ33" s="17"/>
+      <c r="BK33" s="17"/>
+      <c r="BL33" s="17"/>
+      <c r="BM33" s="17"/>
+      <c r="BN33" s="17"/>
+      <c r="BO33" s="17"/>
+      <c r="BP33" s="17"/>
+      <c r="BQ33" s="17"/>
     </row>
-    <row r="34" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>53</v>
       </c>
@@ -37661,57 +37759,81 @@
         <v>12.8326939779569</v>
       </c>
       <c r="M34" s="8"/>
-      <c r="AV34" t="s">
+      <c r="AU34" s="17"/>
+      <c r="AV34" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="AW34">
-        <v>0.48937075406756869</v>
-      </c>
-      <c r="BH34" t="s">
-        <v>42</v>
-      </c>
-      <c r="BI34">
-        <v>0.80843962775308564</v>
-      </c>
+      <c r="AW34" s="21">
+        <v>0.64669026366329108</v>
+      </c>
+      <c r="BE34" s="17"/>
+      <c r="BF34" s="17"/>
+      <c r="BG34" s="17"/>
+      <c r="BH34" s="17"/>
+      <c r="BI34" s="17"/>
+      <c r="BJ34" s="17"/>
+      <c r="BK34" s="17"/>
+      <c r="BL34" s="17"/>
+      <c r="BM34" s="17"/>
+      <c r="BN34" s="17"/>
+      <c r="BO34" s="17"/>
+      <c r="BP34" s="17"/>
+      <c r="BQ34" s="17"/>
     </row>
-    <row r="35" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:69" x14ac:dyDescent="0.25">
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="8"/>
-      <c r="AV35" t="s">
+      <c r="AU35" s="17"/>
+      <c r="AV35" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="AW35">
-        <v>0.23948373493666078</v>
-      </c>
-      <c r="BH35" t="s">
-        <v>45</v>
-      </c>
-      <c r="BI35">
-        <v>0.65357463172154762</v>
-      </c>
+      <c r="AW35" s="21">
+        <v>0.41820829711689689</v>
+      </c>
+      <c r="BE35" s="17"/>
+      <c r="BF35" s="17"/>
+      <c r="BG35" s="17"/>
+      <c r="BH35" s="17"/>
+      <c r="BI35" s="17"/>
+      <c r="BJ35" s="17"/>
+      <c r="BK35" s="17"/>
+      <c r="BL35" s="17"/>
+      <c r="BM35" s="17"/>
+      <c r="BN35" s="17"/>
+      <c r="BO35" s="17"/>
+      <c r="BP35" s="17"/>
+      <c r="BQ35" s="17"/>
     </row>
-    <row r="36" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>72</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8"/>
       <c r="M36" s="8"/>
-      <c r="AV36" t="s">
+      <c r="AU36" s="17"/>
+      <c r="AV36" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="AW36">
-        <v>-1.4021686751118959E-2</v>
-      </c>
-      <c r="BH36" t="s">
-        <v>47</v>
-      </c>
-      <c r="BI36">
-        <v>0.51500448441016666</v>
-      </c>
+      <c r="AW36" s="21">
+        <v>0.18549161596365565</v>
+      </c>
+      <c r="BE36" s="17"/>
+      <c r="BF36" s="17"/>
+      <c r="BG36" s="17"/>
+      <c r="BH36" s="17"/>
+      <c r="BI36" s="17"/>
+      <c r="BJ36" s="17"/>
+      <c r="BK36" s="17"/>
+      <c r="BL36" s="17"/>
+      <c r="BM36" s="17"/>
+      <c r="BN36" s="17"/>
+      <c r="BO36" s="17"/>
+      <c r="BP36" s="17"/>
+      <c r="BQ36" s="17"/>
     </row>
-    <row r="37" spans="1:68" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:69" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>0</v>
       </c>
@@ -37749,20 +37871,28 @@
         <v>11</v>
       </c>
       <c r="M37" s="4"/>
-      <c r="AV37" t="s">
+      <c r="AU37" s="17"/>
+      <c r="AV37" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="AW37">
-        <v>8.1058264596785917E-2</v>
-      </c>
-      <c r="BH37" t="s">
-        <v>49</v>
-      </c>
-      <c r="BI37">
-        <v>2.1354920197063074E-2</v>
-      </c>
+      <c r="AW37" s="21">
+        <v>0.18181409667905082</v>
+      </c>
+      <c r="BE37" s="17"/>
+      <c r="BF37" s="17"/>
+      <c r="BG37" s="17"/>
+      <c r="BH37" s="17"/>
+      <c r="BI37" s="17"/>
+      <c r="BJ37" s="17"/>
+      <c r="BK37" s="17"/>
+      <c r="BL37" s="17"/>
+      <c r="BM37" s="17"/>
+      <c r="BN37" s="17"/>
+      <c r="BO37" s="17"/>
+      <c r="BP37" s="17"/>
+      <c r="BQ37" s="17"/>
     </row>
-    <row r="38" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>17</v>
       </c>
@@ -37801,20 +37931,28 @@
         <v>9.8673684099999903</v>
       </c>
       <c r="M38" s="8"/>
-      <c r="AV38" s="14" t="s">
+      <c r="AU38" s="17"/>
+      <c r="AV38" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="AW38" s="14">
-        <v>9</v>
-      </c>
-      <c r="BH38" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="BI38" s="14">
+      <c r="AW38" s="22">
         <v>8</v>
       </c>
+      <c r="BE38" s="17"/>
+      <c r="BF38" s="17"/>
+      <c r="BG38" s="17"/>
+      <c r="BH38" s="17"/>
+      <c r="BI38" s="17"/>
+      <c r="BJ38" s="17"/>
+      <c r="BK38" s="17"/>
+      <c r="BL38" s="17"/>
+      <c r="BM38" s="17"/>
+      <c r="BN38" s="17"/>
+      <c r="BO38" s="17"/>
+      <c r="BP38" s="17"/>
+      <c r="BQ38" s="17"/>
     </row>
-    <row r="39" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>19</v>
       </c>
@@ -37853,8 +37991,22 @@
         <v>0.16766152125</v>
       </c>
       <c r="M39" s="8"/>
+      <c r="AU39" s="17"/>
+      <c r="BE39" s="17"/>
+      <c r="BF39" s="17"/>
+      <c r="BG39" s="17"/>
+      <c r="BH39" s="17"/>
+      <c r="BI39" s="17"/>
+      <c r="BJ39" s="17"/>
+      <c r="BK39" s="17"/>
+      <c r="BL39" s="17"/>
+      <c r="BM39" s="17"/>
+      <c r="BN39" s="17"/>
+      <c r="BO39" s="17"/>
+      <c r="BP39" s="17"/>
+      <c r="BQ39" s="17"/>
     </row>
-    <row r="40" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>21</v>
       </c>
@@ -37865,7 +38017,7 @@
         <v>0.42964915677977999</v>
       </c>
       <c r="D40" s="6">
-        <v>4.6283799610675601E-2</v>
+        <v>0.146283799610675</v>
       </c>
       <c r="E40" s="7">
         <v>-0.17637365181995501</v>
@@ -37892,14 +38044,25 @@
         <v>0</v>
       </c>
       <c r="M40" s="8"/>
+      <c r="AU40" s="17"/>
       <c r="AV40" t="s">
         <v>54</v>
       </c>
-      <c r="BH40" t="s">
-        <v>54</v>
-      </c>
+      <c r="BE40" s="17"/>
+      <c r="BF40" s="17"/>
+      <c r="BG40" s="17"/>
+      <c r="BH40" s="17"/>
+      <c r="BI40" s="17"/>
+      <c r="BJ40" s="17"/>
+      <c r="BK40" s="17"/>
+      <c r="BL40" s="17"/>
+      <c r="BM40" s="17"/>
+      <c r="BN40" s="17"/>
+      <c r="BO40" s="17"/>
+      <c r="BP40" s="17"/>
+      <c r="BQ40" s="17"/>
     </row>
-    <row r="41" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
@@ -37913,40 +38076,38 @@
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
       <c r="M41" s="8"/>
-      <c r="AV41" s="15"/>
-      <c r="AW41" s="15" t="s">
+      <c r="AU41" s="17"/>
+      <c r="AV41" s="23"/>
+      <c r="AW41" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="AX41" s="15" t="s">
+      <c r="AX41" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="AY41" s="15" t="s">
+      <c r="AY41" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="AZ41" s="15" t="s">
+      <c r="AZ41" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="BA41" s="15" t="s">
+      <c r="BA41" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="BH41" s="15"/>
-      <c r="BI41" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="BJ41" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="BK41" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="BL41" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="BM41" s="15" t="s">
-        <v>59</v>
-      </c>
+      <c r="BE41" s="17"/>
+      <c r="BF41" s="17"/>
+      <c r="BG41" s="17"/>
+      <c r="BH41" s="18"/>
+      <c r="BI41" s="18"/>
+      <c r="BJ41" s="18"/>
+      <c r="BK41" s="18"/>
+      <c r="BL41" s="18"/>
+      <c r="BM41" s="18"/>
+      <c r="BN41" s="17"/>
+      <c r="BO41" s="17"/>
+      <c r="BP41" s="17"/>
+      <c r="BQ41" s="17"/>
     </row>
-    <row r="42" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>26</v>
       </c>
@@ -37979,44 +38140,40 @@
         <v>1.1131942168706099</v>
       </c>
       <c r="M42" s="8"/>
-      <c r="AV42" t="s">
+      <c r="AU42" s="17"/>
+      <c r="AV42" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="AW42">
+      <c r="AW42" s="21">
         <v>2</v>
       </c>
-      <c r="AX42">
-        <v>1.2414046547808623E-2</v>
-      </c>
-      <c r="AY42">
-        <v>6.2070232739043114E-3</v>
-      </c>
-      <c r="AZ42">
-        <v>0.94468880918693632</v>
-      </c>
-      <c r="BA42">
-        <v>0.43987119192687779</v>
-      </c>
-      <c r="BH42" t="s">
-        <v>61</v>
-      </c>
-      <c r="BI42">
-        <v>2</v>
-      </c>
-      <c r="BJ42">
-        <v>4.3018118295363519E-3</v>
-      </c>
-      <c r="BK42">
-        <v>2.150905914768176E-3</v>
-      </c>
-      <c r="BL42">
-        <v>4.7165615711795423</v>
-      </c>
-      <c r="BM42">
-        <v>7.0635694298182949E-2</v>
-      </c>
+      <c r="AX42" s="21">
+        <v>0.11880924359339304</v>
+      </c>
+      <c r="AY42" s="21">
+        <v>5.9404621796696519E-2</v>
+      </c>
+      <c r="AZ42" s="21">
+        <v>1.7970705625589063</v>
+      </c>
+      <c r="BA42" s="21">
+        <v>0.25817774804985977</v>
+      </c>
+      <c r="BE42" s="17"/>
+      <c r="BF42" s="17"/>
+      <c r="BG42" s="17"/>
+      <c r="BH42" s="17"/>
+      <c r="BI42" s="17"/>
+      <c r="BJ42" s="17"/>
+      <c r="BK42" s="17"/>
+      <c r="BL42" s="17"/>
+      <c r="BM42" s="17"/>
+      <c r="BN42" s="17"/>
+      <c r="BO42" s="17"/>
+      <c r="BP42" s="17"/>
+      <c r="BQ42" s="17"/>
     </row>
-    <row r="43" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>25</v>
       </c>
@@ -38053,32 +38210,36 @@
         <v>2.2065870384902602</v>
       </c>
       <c r="M43" s="8"/>
-      <c r="AV43" t="s">
+      <c r="AU43" s="17"/>
+      <c r="AV43" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="AW43">
-        <v>6</v>
-      </c>
-      <c r="AX43">
-        <v>3.9422653556655335E-2</v>
-      </c>
-      <c r="AY43">
-        <v>6.5704422594425561E-3</v>
-      </c>
-      <c r="BH43" t="s">
-        <v>62</v>
-      </c>
-      <c r="BI43">
+      <c r="AW43" s="21">
         <v>5</v>
       </c>
-      <c r="BJ43">
-        <v>2.2801630831146623E-3</v>
-      </c>
-      <c r="BK43">
-        <v>4.5603261662293244E-4</v>
-      </c>
+      <c r="AX43" s="21">
+        <v>0.16528182875609618</v>
+      </c>
+      <c r="AY43" s="21">
+        <v>3.3056365751219237E-2</v>
+      </c>
+      <c r="AZ43" s="21"/>
+      <c r="BA43" s="21"/>
+      <c r="BE43" s="17"/>
+      <c r="BF43" s="17"/>
+      <c r="BG43" s="17"/>
+      <c r="BH43" s="17"/>
+      <c r="BI43" s="17"/>
+      <c r="BJ43" s="17"/>
+      <c r="BK43" s="17"/>
+      <c r="BL43" s="17"/>
+      <c r="BM43" s="17"/>
+      <c r="BN43" s="17"/>
+      <c r="BO43" s="17"/>
+      <c r="BP43" s="17"/>
+      <c r="BQ43" s="17"/>
     </row>
-    <row r="44" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>28</v>
       </c>
@@ -38115,32 +38276,34 @@
         <v>8.4763382350991101</v>
       </c>
       <c r="M44" s="8"/>
-      <c r="AV44" s="14" t="s">
+      <c r="AU44" s="17"/>
+      <c r="AV44" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="AW44" s="14">
-        <v>8</v>
-      </c>
-      <c r="AX44" s="14">
-        <v>5.1836700104463958E-2</v>
-      </c>
-      <c r="AY44" s="14"/>
-      <c r="AZ44" s="14"/>
-      <c r="BA44" s="14"/>
-      <c r="BH44" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="BI44" s="14">
+      <c r="AW44" s="22">
         <v>7</v>
       </c>
-      <c r="BJ44" s="14">
-        <v>6.5819749126510146E-3</v>
-      </c>
-      <c r="BK44" s="14"/>
-      <c r="BL44" s="14"/>
-      <c r="BM44" s="14"/>
+      <c r="AX44" s="22">
+        <v>0.28409107234948922</v>
+      </c>
+      <c r="AY44" s="22"/>
+      <c r="AZ44" s="22"/>
+      <c r="BA44" s="22"/>
+      <c r="BE44" s="17"/>
+      <c r="BF44" s="17"/>
+      <c r="BG44" s="17"/>
+      <c r="BH44" s="17"/>
+      <c r="BI44" s="17"/>
+      <c r="BJ44" s="17"/>
+      <c r="BK44" s="17"/>
+      <c r="BL44" s="17"/>
+      <c r="BM44" s="17"/>
+      <c r="BN44" s="17"/>
+      <c r="BO44" s="17"/>
+      <c r="BP44" s="17"/>
+      <c r="BQ44" s="17"/>
     </row>
-    <row r="45" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>30</v>
       </c>
@@ -38177,8 +38340,22 @@
         <v>9.5412825319663295</v>
       </c>
       <c r="M45" s="8"/>
+      <c r="AU45" s="17"/>
+      <c r="BE45" s="17"/>
+      <c r="BF45" s="17"/>
+      <c r="BG45" s="17"/>
+      <c r="BH45" s="17"/>
+      <c r="BI45" s="17"/>
+      <c r="BJ45" s="17"/>
+      <c r="BK45" s="17"/>
+      <c r="BL45" s="17"/>
+      <c r="BM45" s="17"/>
+      <c r="BN45" s="17"/>
+      <c r="BO45" s="17"/>
+      <c r="BP45" s="17"/>
+      <c r="BQ45" s="17"/>
     </row>
-    <row r="46" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>32</v>
       </c>
@@ -38215,60 +38392,47 @@
         <v>14.7819327483883</v>
       </c>
       <c r="M46" s="8"/>
-      <c r="AV46" s="15"/>
-      <c r="AW46" s="15" t="s">
+      <c r="AU46" s="17"/>
+      <c r="AV46" s="23"/>
+      <c r="AW46" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="AX46" s="15" t="s">
+      <c r="AX46" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="AY46" s="15" t="s">
+      <c r="AY46" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="AZ46" s="15" t="s">
+      <c r="AZ46" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="BA46" s="15" t="s">
+      <c r="BA46" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="BB46" s="15" t="s">
+      <c r="BB46" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="BC46" s="15" t="s">
+      <c r="BC46" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="BD46" s="15" t="s">
+      <c r="BD46" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="BE46" s="16"/>
-      <c r="BF46" s="16"/>
-      <c r="BH46" s="15"/>
-      <c r="BI46" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="BJ46" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="BK46" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="BL46" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="BM46" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="BN46" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="BO46" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="BP46" s="15" t="s">
-        <v>70</v>
-      </c>
+      <c r="BE46" s="18"/>
+      <c r="BF46" s="18"/>
+      <c r="BG46" s="17"/>
+      <c r="BH46" s="18"/>
+      <c r="BI46" s="18"/>
+      <c r="BJ46" s="18"/>
+      <c r="BK46" s="18"/>
+      <c r="BL46" s="18"/>
+      <c r="BM46" s="18"/>
+      <c r="BN46" s="18"/>
+      <c r="BO46" s="18"/>
+      <c r="BP46" s="18"/>
+      <c r="BQ46" s="17"/>
     </row>
-    <row r="47" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>34</v>
       </c>
@@ -38305,183 +38469,144 @@
         <v>48.251680680319097</v>
       </c>
       <c r="M47" s="8"/>
-      <c r="AV47" t="s">
+      <c r="AU47" s="17"/>
+      <c r="AV47" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="AW47">
-        <v>-3.7153468647480391E-2</v>
-      </c>
-      <c r="AX47">
-        <v>0.53084668963576975</v>
-      </c>
-      <c r="AY47">
-        <v>-6.9989074760874043E-2</v>
-      </c>
-      <c r="AZ47">
-        <v>0.94647674698858308</v>
-      </c>
-      <c r="BA47">
-        <v>-1.336088524658321</v>
-      </c>
-      <c r="BB47">
-        <v>1.2617815873633602</v>
-      </c>
-      <c r="BC47">
-        <v>-1.336088524658321</v>
-      </c>
-      <c r="BD47">
-        <v>1.2617815873633602</v>
-      </c>
-      <c r="BH47" t="s">
-        <v>71</v>
-      </c>
-      <c r="BI47">
-        <v>-0.31783730190634446</v>
-      </c>
-      <c r="BJ47">
-        <v>0.13933086421503724</v>
-      </c>
-      <c r="BK47">
-        <v>-2.2811693855268715</v>
-      </c>
-      <c r="BL47">
-        <v>7.1433539506165974E-2</v>
-      </c>
-      <c r="BM47">
-        <v>-0.67599869060102902</v>
-      </c>
-      <c r="BN47">
-        <v>4.0324086788340097E-2</v>
-      </c>
-      <c r="BO47">
-        <v>-0.67599869060102902</v>
-      </c>
-      <c r="BP47">
-        <v>4.0324086788340097E-2</v>
-      </c>
+      <c r="AW47" s="21">
+        <v>-1.195315653107293</v>
+      </c>
+      <c r="AX47" s="21">
+        <v>1.191608537898637</v>
+      </c>
+      <c r="AY47" s="21">
+        <v>-1.0031110176628923</v>
+      </c>
+      <c r="AZ47" s="21">
+        <v>0.36185273760739334</v>
+      </c>
+      <c r="BA47" s="21">
+        <v>-4.2584429158186765</v>
+      </c>
+      <c r="BB47" s="21">
+        <v>1.8678116096040904</v>
+      </c>
+      <c r="BC47" s="21">
+        <v>-4.2584429158186765</v>
+      </c>
+      <c r="BD47" s="21">
+        <v>1.8678116096040904</v>
+      </c>
+      <c r="BE47" s="17"/>
+      <c r="BF47" s="17"/>
+      <c r="BG47" s="17"/>
+      <c r="BH47" s="17"/>
+      <c r="BI47" s="17"/>
+      <c r="BJ47" s="17"/>
+      <c r="BK47" s="17"/>
+      <c r="BL47" s="17"/>
+      <c r="BM47" s="17"/>
+      <c r="BN47" s="17"/>
+      <c r="BO47" s="17"/>
+      <c r="BP47" s="17"/>
+      <c r="BQ47" s="17"/>
     </row>
-    <row r="48" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:69" x14ac:dyDescent="0.25">
       <c r="K48" s="8"/>
       <c r="L48" s="8"/>
       <c r="M48" s="8"/>
-      <c r="AV48" t="s">
+      <c r="AU48" s="17"/>
+      <c r="AV48" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AW48">
-        <v>0.15629388026054086</v>
-      </c>
-      <c r="AX48">
-        <v>0.50694423610723038</v>
-      </c>
-      <c r="AY48">
-        <v>0.30830586310775432</v>
-      </c>
-      <c r="AZ48">
-        <v>0.76827290458907793</v>
-      </c>
-      <c r="BA48">
-        <v>-1.0841539789398749</v>
-      </c>
-      <c r="BB48">
-        <v>1.3967417394609567</v>
-      </c>
-      <c r="BC48">
-        <v>-1.0841539789398749</v>
-      </c>
-      <c r="BD48">
-        <v>1.3967417394609567</v>
-      </c>
-      <c r="BH48" t="s">
-        <v>5</v>
-      </c>
-      <c r="BI48">
-        <v>0.39577834821354096</v>
-      </c>
-      <c r="BJ48">
-        <v>0.13351643930761767</v>
-      </c>
-      <c r="BK48">
-        <v>2.9642667993989873</v>
-      </c>
-      <c r="BL48">
-        <v>3.13639480730745E-2</v>
-      </c>
-      <c r="BM48">
-        <v>5.2563414570540479E-2</v>
-      </c>
-      <c r="BN48">
-        <v>0.73899328185654145</v>
-      </c>
-      <c r="BO48">
-        <v>5.2563414570540479E-2</v>
-      </c>
-      <c r="BP48">
-        <v>0.73899328185654145</v>
-      </c>
+      <c r="AW48" s="21">
+        <v>0.94235237879801748</v>
+      </c>
+      <c r="AX48" s="21">
+        <v>1.1365443595336113</v>
+      </c>
+      <c r="AY48" s="21">
+        <v>0.82913823019166466</v>
+      </c>
+      <c r="AZ48" s="21">
+        <v>0.44479191524306583</v>
+      </c>
+      <c r="BA48" s="21">
+        <v>-1.9792279072139931</v>
+      </c>
+      <c r="BB48" s="21">
+        <v>3.8639326648100281</v>
+      </c>
+      <c r="BC48" s="21">
+        <v>-1.9792279072139931</v>
+      </c>
+      <c r="BD48" s="21">
+        <v>3.8639326648100281</v>
+      </c>
+      <c r="BE48" s="17"/>
+      <c r="BF48" s="17"/>
+      <c r="BG48" s="17"/>
+      <c r="BH48" s="17"/>
+      <c r="BI48" s="17"/>
+      <c r="BJ48" s="17"/>
+      <c r="BK48" s="17"/>
+      <c r="BL48" s="17"/>
+      <c r="BM48" s="17"/>
+      <c r="BN48" s="17"/>
+      <c r="BO48" s="17"/>
+      <c r="BP48" s="17"/>
+      <c r="BQ48" s="17"/>
     </row>
-    <row r="49" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:69" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>73</v>
       </c>
       <c r="K49" s="8"/>
       <c r="L49" s="8"/>
       <c r="M49" s="8"/>
-      <c r="AV49" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="AW49" s="14">
-        <v>-4.5755113050218923E-3</v>
-      </c>
-      <c r="AX49" s="14">
-        <v>3.3660004022408939E-3</v>
-      </c>
-      <c r="AY49" s="14">
-        <v>-1.3593317760674579</v>
-      </c>
-      <c r="AZ49" s="14">
-        <v>0.22290940119196909</v>
-      </c>
-      <c r="BA49" s="14">
-        <v>-1.281181758022387E-2</v>
-      </c>
-      <c r="BB49" s="14">
-        <v>3.6607949701800858E-3</v>
-      </c>
-      <c r="BC49" s="14">
-        <v>-1.281181758022387E-2</v>
-      </c>
-      <c r="BD49" s="14">
-        <v>3.6607949701800858E-3</v>
-      </c>
-      <c r="BH49" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="BI49" s="14">
-        <v>-1.0372276668328196E-3</v>
-      </c>
-      <c r="BJ49" s="14">
-        <v>8.7477052432087445E-4</v>
-      </c>
-      <c r="BK49" s="14">
-        <v>-1.1857140106979123</v>
-      </c>
-      <c r="BL49" s="14">
-        <v>0.28900777821946655</v>
-      </c>
-      <c r="BM49" s="14">
-        <v>-3.2858968870021149E-3</v>
-      </c>
-      <c r="BN49" s="14">
-        <v>1.2114415533364755E-3</v>
-      </c>
-      <c r="BO49" s="14">
-        <v>-3.2858968870021149E-3</v>
-      </c>
-      <c r="BP49" s="14">
-        <v>1.2114415533364755E-3</v>
-      </c>
+      <c r="AU49" s="17"/>
+      <c r="AV49" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="AW49" s="22">
+        <v>-3.3769292142629526E-2</v>
+      </c>
+      <c r="AX49" s="22">
+        <v>2.0523635794965786E-2</v>
+      </c>
+      <c r="AY49" s="22">
+        <v>-1.6453854706831597</v>
+      </c>
+      <c r="AZ49" s="22">
+        <v>0.16080946538808036</v>
+      </c>
+      <c r="BA49" s="22">
+        <v>-8.6526977518383855E-2</v>
+      </c>
+      <c r="BB49" s="22">
+        <v>1.8988393233124803E-2</v>
+      </c>
+      <c r="BC49" s="22">
+        <v>-8.6526977518383855E-2</v>
+      </c>
+      <c r="BD49" s="22">
+        <v>1.8988393233124803E-2</v>
+      </c>
+      <c r="BE49" s="17"/>
+      <c r="BF49" s="17"/>
+      <c r="BG49" s="17"/>
+      <c r="BH49" s="17"/>
+      <c r="BI49" s="17"/>
+      <c r="BJ49" s="17"/>
+      <c r="BK49" s="17"/>
+      <c r="BL49" s="17"/>
+      <c r="BM49" s="17"/>
+      <c r="BN49" s="17"/>
+      <c r="BO49" s="17"/>
+      <c r="BP49" s="17"/>
+      <c r="BQ49" s="17"/>
     </row>
-    <row r="50" spans="1:68" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:69" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>0</v>
       </c>
@@ -38519,14 +38644,22 @@
         <v>11</v>
       </c>
       <c r="M50" s="4"/>
-      <c r="AV50" t="s">
-        <v>74</v>
-      </c>
-      <c r="BH50" t="s">
-        <v>74</v>
-      </c>
+      <c r="AU50" s="17"/>
+      <c r="BE50" s="17"/>
+      <c r="BF50" s="17"/>
+      <c r="BG50" s="17"/>
+      <c r="BH50" s="17"/>
+      <c r="BI50" s="17"/>
+      <c r="BJ50" s="17"/>
+      <c r="BK50" s="17"/>
+      <c r="BL50" s="17"/>
+      <c r="BM50" s="17"/>
+      <c r="BN50" s="17"/>
+      <c r="BO50" s="17"/>
+      <c r="BP50" s="17"/>
+      <c r="BQ50" s="17"/>
     </row>
-    <row r="51" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>17</v>
       </c>
@@ -38565,8 +38698,22 @@
         <v>9.8673684099999903</v>
       </c>
       <c r="M51" s="8"/>
+      <c r="AU51" s="17"/>
+      <c r="BE51" s="17"/>
+      <c r="BF51" s="17"/>
+      <c r="BG51" s="17"/>
+      <c r="BH51" s="17"/>
+      <c r="BI51" s="17"/>
+      <c r="BJ51" s="17"/>
+      <c r="BK51" s="17"/>
+      <c r="BL51" s="17"/>
+      <c r="BM51" s="17"/>
+      <c r="BN51" s="17"/>
+      <c r="BO51" s="17"/>
+      <c r="BP51" s="17"/>
+      <c r="BQ51" s="17"/>
     </row>
-    <row r="52" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>19</v>
       </c>
@@ -38605,16 +38752,22 @@
         <v>0.16766152125</v>
       </c>
       <c r="M52" s="8"/>
-      <c r="AV52" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="AW52" s="12"/>
-      <c r="BH52" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="BI52" s="12"/>
+      <c r="AU52" s="17"/>
+      <c r="BE52" s="17"/>
+      <c r="BF52" s="17"/>
+      <c r="BG52" s="17"/>
+      <c r="BH52" s="19"/>
+      <c r="BI52" s="19"/>
+      <c r="BJ52" s="17"/>
+      <c r="BK52" s="17"/>
+      <c r="BL52" s="17"/>
+      <c r="BM52" s="17"/>
+      <c r="BN52" s="17"/>
+      <c r="BO52" s="17"/>
+      <c r="BP52" s="17"/>
+      <c r="BQ52" s="17"/>
     </row>
-    <row r="53" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>21</v>
       </c>
@@ -38652,20 +38805,31 @@
         <v>0</v>
       </c>
       <c r="M53" s="8"/>
-      <c r="AV53" t="s">
-        <v>42</v>
-      </c>
-      <c r="AW53">
-        <v>0.84932579024205879</v>
-      </c>
-      <c r="BH53" t="s">
-        <v>42</v>
-      </c>
-      <c r="BI53">
-        <v>0.91216011160202104</v>
-      </c>
+      <c r="AU53" s="17"/>
+      <c r="AV53" s="17"/>
+      <c r="AW53" s="17"/>
+      <c r="AX53" s="17"/>
+      <c r="AY53" s="17"/>
+      <c r="AZ53" s="17"/>
+      <c r="BA53" s="17"/>
+      <c r="BB53" s="17"/>
+      <c r="BC53" s="17"/>
+      <c r="BD53" s="17"/>
+      <c r="BE53" s="17"/>
+      <c r="BF53" s="17"/>
+      <c r="BG53" s="17"/>
+      <c r="BH53" s="17"/>
+      <c r="BI53" s="17"/>
+      <c r="BJ53" s="17"/>
+      <c r="BK53" s="17"/>
+      <c r="BL53" s="17"/>
+      <c r="BM53" s="17"/>
+      <c r="BN53" s="17"/>
+      <c r="BO53" s="17"/>
+      <c r="BP53" s="17"/>
+      <c r="BQ53" s="17"/>
     </row>
-    <row r="54" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
@@ -38679,20 +38843,31 @@
       <c r="K54" s="8"/>
       <c r="L54" s="8"/>
       <c r="M54" s="8"/>
-      <c r="AV54" t="s">
-        <v>45</v>
-      </c>
-      <c r="AW54">
-        <v>0.7213542979702976</v>
-      </c>
-      <c r="BH54" t="s">
-        <v>45</v>
-      </c>
-      <c r="BI54">
-        <v>0.83203606919781148</v>
-      </c>
+      <c r="AU54" s="17"/>
+      <c r="AV54" s="17"/>
+      <c r="AW54" s="17"/>
+      <c r="AX54" s="17"/>
+      <c r="AY54" s="17"/>
+      <c r="AZ54" s="17"/>
+      <c r="BA54" s="17"/>
+      <c r="BB54" s="17"/>
+      <c r="BC54" s="17"/>
+      <c r="BD54" s="17"/>
+      <c r="BE54" s="17"/>
+      <c r="BF54" s="17"/>
+      <c r="BG54" s="17"/>
+      <c r="BH54" s="17"/>
+      <c r="BI54" s="17"/>
+      <c r="BJ54" s="17"/>
+      <c r="BK54" s="17"/>
+      <c r="BL54" s="17"/>
+      <c r="BM54" s="17"/>
+      <c r="BN54" s="17"/>
+      <c r="BO54" s="17"/>
+      <c r="BP54" s="17"/>
+      <c r="BQ54" s="17"/>
     </row>
-    <row r="55" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>40</v>
       </c>
@@ -38730,20 +38905,31 @@
         <v>1.1131942168706099</v>
       </c>
       <c r="M55" s="8"/>
-      <c r="AV55" t="s">
-        <v>47</v>
-      </c>
-      <c r="AW55">
-        <v>0.62847239729373017</v>
-      </c>
-      <c r="BH55" t="s">
-        <v>47</v>
-      </c>
-      <c r="BI55">
-        <v>0.76485049687693607</v>
-      </c>
+      <c r="AU55" s="17"/>
+      <c r="AV55" s="17"/>
+      <c r="AW55" s="17"/>
+      <c r="AX55" s="17"/>
+      <c r="AY55" s="17"/>
+      <c r="AZ55" s="17"/>
+      <c r="BA55" s="17"/>
+      <c r="BB55" s="17"/>
+      <c r="BC55" s="17"/>
+      <c r="BD55" s="17"/>
+      <c r="BE55" s="17"/>
+      <c r="BF55" s="17"/>
+      <c r="BG55" s="17"/>
+      <c r="BH55" s="17"/>
+      <c r="BI55" s="17"/>
+      <c r="BJ55" s="17"/>
+      <c r="BK55" s="17"/>
+      <c r="BL55" s="17"/>
+      <c r="BM55" s="17"/>
+      <c r="BN55" s="17"/>
+      <c r="BO55" s="17"/>
+      <c r="BP55" s="17"/>
+      <c r="BQ55" s="17"/>
     </row>
-    <row r="56" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>43</v>
       </c>
@@ -38781,20 +38967,31 @@
         <v>8.4763382350991101</v>
       </c>
       <c r="M56" s="8"/>
-      <c r="AV56" t="s">
-        <v>49</v>
-      </c>
-      <c r="AW56">
-        <v>4.9064708449678154E-2</v>
-      </c>
-      <c r="BH56" t="s">
-        <v>49</v>
-      </c>
-      <c r="BI56">
-        <v>1.4869662933437701E-2</v>
-      </c>
+      <c r="AU56" s="17"/>
+      <c r="AV56" s="17"/>
+      <c r="AW56" s="17"/>
+      <c r="AX56" s="17"/>
+      <c r="AY56" s="17"/>
+      <c r="AZ56" s="17"/>
+      <c r="BA56" s="17"/>
+      <c r="BB56" s="17"/>
+      <c r="BC56" s="17"/>
+      <c r="BD56" s="17"/>
+      <c r="BE56" s="17"/>
+      <c r="BF56" s="17"/>
+      <c r="BG56" s="17"/>
+      <c r="BH56" s="17"/>
+      <c r="BI56" s="17"/>
+      <c r="BJ56" s="17"/>
+      <c r="BK56" s="17"/>
+      <c r="BL56" s="17"/>
+      <c r="BM56" s="17"/>
+      <c r="BN56" s="17"/>
+      <c r="BO56" s="17"/>
+      <c r="BP56" s="17"/>
+      <c r="BQ56" s="17"/>
     </row>
-    <row r="57" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>46</v>
       </c>
@@ -38832,20 +39029,31 @@
         <v>9.5412825319663295</v>
       </c>
       <c r="M57" s="8"/>
-      <c r="AV57" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="AW57" s="14">
-        <v>9</v>
-      </c>
-      <c r="BH57" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="BI57" s="14">
-        <v>8</v>
-      </c>
+      <c r="AU57" s="17"/>
+      <c r="AV57" s="17"/>
+      <c r="AW57" s="17"/>
+      <c r="AX57" s="17"/>
+      <c r="AY57" s="17"/>
+      <c r="AZ57" s="17"/>
+      <c r="BA57" s="17"/>
+      <c r="BB57" s="17"/>
+      <c r="BC57" s="17"/>
+      <c r="BD57" s="17"/>
+      <c r="BE57" s="17"/>
+      <c r="BF57" s="17"/>
+      <c r="BG57" s="17"/>
+      <c r="BH57" s="17"/>
+      <c r="BI57" s="17"/>
+      <c r="BJ57" s="17"/>
+      <c r="BK57" s="17"/>
+      <c r="BL57" s="17"/>
+      <c r="BM57" s="17"/>
+      <c r="BN57" s="17"/>
+      <c r="BO57" s="17"/>
+      <c r="BP57" s="17"/>
+      <c r="BQ57" s="17"/>
     </row>
-    <row r="58" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>48</v>
       </c>
@@ -38883,8 +39091,31 @@
         <v>14.7819327483883</v>
       </c>
       <c r="M58" s="8"/>
+      <c r="AU58" s="17"/>
+      <c r="AV58" s="17"/>
+      <c r="AW58" s="17"/>
+      <c r="AX58" s="17"/>
+      <c r="AY58" s="17"/>
+      <c r="AZ58" s="17"/>
+      <c r="BA58" s="17"/>
+      <c r="BB58" s="17"/>
+      <c r="BC58" s="17"/>
+      <c r="BD58" s="17"/>
+      <c r="BE58" s="17"/>
+      <c r="BF58" s="17"/>
+      <c r="BG58" s="17"/>
+      <c r="BH58" s="17"/>
+      <c r="BI58" s="17"/>
+      <c r="BJ58" s="17"/>
+      <c r="BK58" s="17"/>
+      <c r="BL58" s="17"/>
+      <c r="BM58" s="17"/>
+      <c r="BN58" s="17"/>
+      <c r="BO58" s="17"/>
+      <c r="BP58" s="17"/>
+      <c r="BQ58" s="17"/>
     </row>
-    <row r="59" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>50</v>
       </c>
@@ -38922,14 +39153,31 @@
         <v>15.671540073004801</v>
       </c>
       <c r="M59" s="8"/>
-      <c r="AV59" t="s">
-        <v>54</v>
-      </c>
-      <c r="BH59" t="s">
-        <v>54</v>
-      </c>
+      <c r="AU59" s="17"/>
+      <c r="AV59" s="17"/>
+      <c r="AW59" s="17"/>
+      <c r="AX59" s="17"/>
+      <c r="AY59" s="17"/>
+      <c r="AZ59" s="17"/>
+      <c r="BA59" s="17"/>
+      <c r="BB59" s="17"/>
+      <c r="BC59" s="17"/>
+      <c r="BD59" s="17"/>
+      <c r="BE59" s="17"/>
+      <c r="BF59" s="17"/>
+      <c r="BG59" s="17"/>
+      <c r="BH59" s="17"/>
+      <c r="BI59" s="17"/>
+      <c r="BJ59" s="17"/>
+      <c r="BK59" s="17"/>
+      <c r="BL59" s="17"/>
+      <c r="BM59" s="17"/>
+      <c r="BN59" s="17"/>
+      <c r="BO59" s="17"/>
+      <c r="BP59" s="17"/>
+      <c r="BQ59" s="17"/>
     </row>
-    <row r="60" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>52</v>
       </c>
@@ -38967,40 +39215,31 @@
         <v>48.251680680319097</v>
       </c>
       <c r="M60" s="8"/>
-      <c r="AV60" s="15"/>
-      <c r="AW60" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="AX60" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="AY60" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="AZ60" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="BA60" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="BH60" s="15"/>
-      <c r="BI60" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="BJ60" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="BK60" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="BL60" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="BM60" s="15" t="s">
-        <v>59</v>
-      </c>
+      <c r="AU60" s="17"/>
+      <c r="AV60" s="18"/>
+      <c r="AW60" s="18"/>
+      <c r="AX60" s="18"/>
+      <c r="AY60" s="18"/>
+      <c r="AZ60" s="18"/>
+      <c r="BA60" s="18"/>
+      <c r="BB60" s="17"/>
+      <c r="BC60" s="17"/>
+      <c r="BD60" s="17"/>
+      <c r="BE60" s="17"/>
+      <c r="BF60" s="17"/>
+      <c r="BG60" s="17"/>
+      <c r="BH60" s="18"/>
+      <c r="BI60" s="18"/>
+      <c r="BJ60" s="18"/>
+      <c r="BK60" s="18"/>
+      <c r="BL60" s="18"/>
+      <c r="BM60" s="18"/>
+      <c r="BN60" s="17"/>
+      <c r="BO60" s="17"/>
+      <c r="BP60" s="17"/>
+      <c r="BQ60" s="17"/>
     </row>
-    <row r="61" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>53</v>
       </c>
@@ -39038,105 +39277,90 @@
         <v>12.8326939779569</v>
       </c>
       <c r="M61" s="8"/>
-      <c r="AV61" t="s">
-        <v>61</v>
-      </c>
-      <c r="AW61">
-        <v>2</v>
-      </c>
-      <c r="AX61">
-        <v>3.7392626412952448E-2</v>
-      </c>
-      <c r="AY61">
-        <v>1.8696313206476224E-2</v>
-      </c>
-      <c r="AZ61">
-        <v>7.7663602135166334</v>
-      </c>
-      <c r="BA61">
-        <v>2.1635007296750559E-2</v>
-      </c>
-      <c r="BH61" t="s">
-        <v>61</v>
-      </c>
-      <c r="BI61">
-        <v>2</v>
-      </c>
-      <c r="BJ61">
-        <v>5.4764405338807581E-3</v>
-      </c>
-      <c r="BK61">
-        <v>2.7382202669403791E-3</v>
-      </c>
-      <c r="BL61">
-        <v>12.384147971889607</v>
-      </c>
-      <c r="BM61">
-        <v>1.1562189268396628E-2</v>
-      </c>
+      <c r="AU61" s="17"/>
+      <c r="AV61" s="17"/>
+      <c r="AW61" s="17"/>
+      <c r="AX61" s="17"/>
+      <c r="AY61" s="17"/>
+      <c r="AZ61" s="17"/>
+      <c r="BA61" s="17"/>
+      <c r="BB61" s="17"/>
+      <c r="BC61" s="17"/>
+      <c r="BD61" s="17"/>
+      <c r="BE61" s="17"/>
+      <c r="BF61" s="17"/>
+      <c r="BG61" s="17"/>
+      <c r="BH61" s="17"/>
+      <c r="BI61" s="17"/>
+      <c r="BJ61" s="17"/>
+      <c r="BK61" s="17"/>
+      <c r="BL61" s="17"/>
+      <c r="BM61" s="17"/>
+      <c r="BN61" s="17"/>
+      <c r="BO61" s="17"/>
+      <c r="BP61" s="17"/>
+      <c r="BQ61" s="17"/>
     </row>
-    <row r="62" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:69" x14ac:dyDescent="0.25">
       <c r="K62" s="8"/>
       <c r="L62" s="8"/>
       <c r="M62" s="8"/>
-      <c r="AV62" t="s">
-        <v>62</v>
-      </c>
-      <c r="AW62">
-        <v>6</v>
-      </c>
-      <c r="AX62">
-        <v>1.4444073691511513E-2</v>
-      </c>
-      <c r="AY62">
-        <v>2.4073456152519188E-3</v>
-      </c>
-      <c r="BH62" t="s">
-        <v>62</v>
-      </c>
-      <c r="BI62">
-        <v>5</v>
-      </c>
-      <c r="BJ62">
-        <v>1.1055343787702554E-3</v>
-      </c>
-      <c r="BK62">
-        <v>2.2110687575405109E-4</v>
-      </c>
+      <c r="AU62" s="17"/>
+      <c r="AV62" s="17"/>
+      <c r="AW62" s="17"/>
+      <c r="AX62" s="17"/>
+      <c r="AY62" s="17"/>
+      <c r="AZ62" s="17"/>
+      <c r="BA62" s="17"/>
+      <c r="BB62" s="17"/>
+      <c r="BC62" s="17"/>
+      <c r="BD62" s="17"/>
+      <c r="BE62" s="17"/>
+      <c r="BF62" s="17"/>
+      <c r="BG62" s="17"/>
+      <c r="BH62" s="17"/>
+      <c r="BI62" s="17"/>
+      <c r="BJ62" s="17"/>
+      <c r="BK62" s="17"/>
+      <c r="BL62" s="17"/>
+      <c r="BM62" s="17"/>
+      <c r="BN62" s="17"/>
+      <c r="BO62" s="17"/>
+      <c r="BP62" s="17"/>
+      <c r="BQ62" s="17"/>
     </row>
-    <row r="63" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>75</v>
       </c>
       <c r="K63" s="8"/>
       <c r="L63" s="8"/>
       <c r="M63" s="8"/>
-      <c r="AV63" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="AW63" s="14">
-        <v>8</v>
-      </c>
-      <c r="AX63" s="14">
-        <v>5.1836700104463965E-2</v>
-      </c>
-      <c r="AY63" s="14"/>
-      <c r="AZ63" s="14"/>
-      <c r="BA63" s="14"/>
-      <c r="BH63" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="BI63" s="14">
-        <v>7</v>
-      </c>
-      <c r="BJ63" s="14">
-        <v>6.5819749126510138E-3</v>
-      </c>
-      <c r="BK63" s="14"/>
-      <c r="BL63" s="14"/>
-      <c r="BM63" s="14"/>
+      <c r="AU63" s="17"/>
+      <c r="AV63" s="17"/>
+      <c r="AW63" s="17"/>
+      <c r="AX63" s="17"/>
+      <c r="AY63" s="17"/>
+      <c r="AZ63" s="17"/>
+      <c r="BA63" s="17"/>
+      <c r="BB63" s="17"/>
+      <c r="BC63" s="17"/>
+      <c r="BD63" s="17"/>
+      <c r="BE63" s="17"/>
+      <c r="BF63" s="17"/>
+      <c r="BG63" s="17"/>
+      <c r="BH63" s="17"/>
+      <c r="BI63" s="17"/>
+      <c r="BJ63" s="17"/>
+      <c r="BK63" s="17"/>
+      <c r="BL63" s="17"/>
+      <c r="BM63" s="17"/>
+      <c r="BN63" s="17"/>
+      <c r="BO63" s="17"/>
+      <c r="BP63" s="17"/>
+      <c r="BQ63" s="17"/>
     </row>
-    <row r="64" spans="1:68" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:69" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>0</v>
       </c>
@@ -39174,8 +39398,31 @@
         <v>11</v>
       </c>
       <c r="M64" s="4"/>
+      <c r="AU64" s="17"/>
+      <c r="AV64" s="17"/>
+      <c r="AW64" s="17"/>
+      <c r="AX64" s="17"/>
+      <c r="AY64" s="17"/>
+      <c r="AZ64" s="17"/>
+      <c r="BA64" s="17"/>
+      <c r="BB64" s="17"/>
+      <c r="BC64" s="17"/>
+      <c r="BD64" s="17"/>
+      <c r="BE64" s="17"/>
+      <c r="BF64" s="17"/>
+      <c r="BG64" s="17"/>
+      <c r="BH64" s="17"/>
+      <c r="BI64" s="17"/>
+      <c r="BJ64" s="17"/>
+      <c r="BK64" s="17"/>
+      <c r="BL64" s="17"/>
+      <c r="BM64" s="17"/>
+      <c r="BN64" s="17"/>
+      <c r="BO64" s="17"/>
+      <c r="BP64" s="17"/>
+      <c r="BQ64" s="17"/>
     </row>
-    <row r="65" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>17</v>
       </c>
@@ -39215,60 +39462,31 @@
         <v>9.8673684099999903</v>
       </c>
       <c r="M65" s="8"/>
-      <c r="AV65" s="15"/>
-      <c r="AW65" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="AX65" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="AY65" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="AZ65" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="BA65" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB65" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="BC65" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="BD65" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="BE65" s="16"/>
-      <c r="BF65" s="16"/>
-      <c r="BH65" s="15"/>
-      <c r="BI65" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="BJ65" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="BK65" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="BL65" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="BM65" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="BN65" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="BO65" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="BP65" s="15" t="s">
-        <v>70</v>
-      </c>
+      <c r="AU65" s="17"/>
+      <c r="AV65" s="18"/>
+      <c r="AW65" s="18"/>
+      <c r="AX65" s="18"/>
+      <c r="AY65" s="18"/>
+      <c r="AZ65" s="18"/>
+      <c r="BA65" s="18"/>
+      <c r="BB65" s="18"/>
+      <c r="BC65" s="18"/>
+      <c r="BD65" s="18"/>
+      <c r="BE65" s="18"/>
+      <c r="BF65" s="18"/>
+      <c r="BG65" s="17"/>
+      <c r="BH65" s="18"/>
+      <c r="BI65" s="18"/>
+      <c r="BJ65" s="18"/>
+      <c r="BK65" s="18"/>
+      <c r="BL65" s="18"/>
+      <c r="BM65" s="18"/>
+      <c r="BN65" s="18"/>
+      <c r="BO65" s="18"/>
+      <c r="BP65" s="18"/>
+      <c r="BQ65" s="17"/>
     </row>
-    <row r="66" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>19</v>
       </c>
@@ -39308,62 +39526,31 @@
         <v>0.16766152125</v>
       </c>
       <c r="M66" s="8"/>
-      <c r="AV66" t="s">
-        <v>71</v>
-      </c>
-      <c r="AW66">
-        <v>-0.21589435791032491</v>
-      </c>
-      <c r="AX66">
-        <v>0.32480924299683162</v>
-      </c>
-      <c r="AY66">
-        <v>-0.66468046265675662</v>
-      </c>
-      <c r="AZ66">
-        <v>0.5309563140617849</v>
-      </c>
-      <c r="BA66">
-        <v>-1.0106739439606984</v>
-      </c>
-      <c r="BB66">
-        <v>0.57888522814004872</v>
-      </c>
-      <c r="BC66">
-        <v>-1.0106739439606984</v>
-      </c>
-      <c r="BD66">
-        <v>0.57888522814004872</v>
-      </c>
-      <c r="BH66" t="s">
-        <v>71</v>
-      </c>
-      <c r="BI66">
-        <v>-0.32738206045642781</v>
-      </c>
-      <c r="BJ66">
-        <v>9.706802832371221E-2</v>
-      </c>
-      <c r="BK66">
-        <v>-3.3727074311702432</v>
-      </c>
-      <c r="BL66">
-        <v>1.9831094741875301E-2</v>
-      </c>
-      <c r="BM66">
-        <v>-0.57690337088639376</v>
-      </c>
-      <c r="BN66">
-        <v>-7.7860750026461867E-2</v>
-      </c>
-      <c r="BO66">
-        <v>-0.57690337088639376</v>
-      </c>
-      <c r="BP66">
-        <v>-7.7860750026461867E-2</v>
-      </c>
+      <c r="AU66" s="17"/>
+      <c r="AV66" s="17"/>
+      <c r="AW66" s="17"/>
+      <c r="AX66" s="17"/>
+      <c r="AY66" s="17"/>
+      <c r="AZ66" s="17"/>
+      <c r="BA66" s="17"/>
+      <c r="BB66" s="17"/>
+      <c r="BC66" s="17"/>
+      <c r="BD66" s="17"/>
+      <c r="BE66" s="17"/>
+      <c r="BF66" s="17"/>
+      <c r="BG66" s="17"/>
+      <c r="BH66" s="17"/>
+      <c r="BI66" s="17"/>
+      <c r="BJ66" s="17"/>
+      <c r="BK66" s="17"/>
+      <c r="BL66" s="17"/>
+      <c r="BM66" s="17"/>
+      <c r="BN66" s="17"/>
+      <c r="BO66" s="17"/>
+      <c r="BP66" s="17"/>
+      <c r="BQ66" s="17"/>
     </row>
-    <row r="67" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>23</v>
       </c>
@@ -39401,62 +39588,31 @@
         <v>0</v>
       </c>
       <c r="M67" s="8"/>
-      <c r="AV67" t="s">
-        <v>5</v>
-      </c>
-      <c r="AW67">
-        <v>0.43275382393399581</v>
-      </c>
-      <c r="AX67">
-        <v>0.3172485846531849</v>
-      </c>
-      <c r="AY67">
-        <v>1.3640843328176888</v>
-      </c>
-      <c r="AZ67">
-        <v>0.22149192279350693</v>
-      </c>
-      <c r="BA67">
-        <v>-0.34352549761285051</v>
-      </c>
-      <c r="BB67">
-        <v>1.2090331454808421</v>
-      </c>
-      <c r="BC67">
-        <v>-0.34352549761285051</v>
-      </c>
-      <c r="BD67">
-        <v>1.2090331454808421</v>
-      </c>
-      <c r="BH67" t="s">
-        <v>5</v>
-      </c>
-      <c r="BI67">
-        <v>0.37057009676235214</v>
-      </c>
-      <c r="BJ67">
-        <v>9.2178985676072869E-2</v>
-      </c>
-      <c r="BK67">
-        <v>4.0201147153492922</v>
-      </c>
-      <c r="BL67">
-        <v>1.0119639985013064E-2</v>
-      </c>
-      <c r="BM67">
-        <v>0.13361647055605916</v>
-      </c>
-      <c r="BN67">
-        <v>0.6075237229686451</v>
-      </c>
-      <c r="BO67">
-        <v>0.13361647055605916</v>
-      </c>
-      <c r="BP67">
-        <v>0.6075237229686451</v>
-      </c>
+      <c r="AU67" s="17"/>
+      <c r="AV67" s="17"/>
+      <c r="AW67" s="17"/>
+      <c r="AX67" s="17"/>
+      <c r="AY67" s="17"/>
+      <c r="AZ67" s="17"/>
+      <c r="BA67" s="17"/>
+      <c r="BB67" s="17"/>
+      <c r="BC67" s="17"/>
+      <c r="BD67" s="17"/>
+      <c r="BE67" s="17"/>
+      <c r="BF67" s="17"/>
+      <c r="BG67" s="17"/>
+      <c r="BH67" s="17"/>
+      <c r="BI67" s="17"/>
+      <c r="BJ67" s="17"/>
+      <c r="BK67" s="17"/>
+      <c r="BL67" s="17"/>
+      <c r="BM67" s="17"/>
+      <c r="BN67" s="17"/>
+      <c r="BO67" s="17"/>
+      <c r="BP67" s="17"/>
+      <c r="BQ67" s="17"/>
     </row>
-    <row r="68" spans="1:68" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
       <c r="B68" s="7"/>
       <c r="C68" s="7"/>
@@ -39470,62 +39626,31 @@
       <c r="K68" s="8"/>
       <c r="L68" s="8"/>
       <c r="M68" s="8"/>
-      <c r="AV68" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="AW68" s="14">
-        <v>-0.535089924150702</v>
-      </c>
-      <c r="AX68" s="14">
-        <v>0.13626864204884859</v>
-      </c>
-      <c r="AY68" s="14">
-        <v>-3.9267282340634675</v>
-      </c>
-      <c r="AZ68" s="14">
-        <v>7.741818907155102E-3</v>
-      </c>
-      <c r="BA68" s="14">
-        <v>-0.86852727931946139</v>
-      </c>
-      <c r="BB68" s="14">
-        <v>-0.20165256898194267</v>
-      </c>
-      <c r="BC68" s="14">
-        <v>-0.86852727931946139</v>
-      </c>
-      <c r="BD68" s="14">
-        <v>-0.20165256898194267</v>
-      </c>
-      <c r="BH68" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="BI68" s="14">
-        <v>7.8723011754401689E-2</v>
-      </c>
-      <c r="BJ68" s="14">
-        <v>2.7470846564143551E-2</v>
-      </c>
-      <c r="BK68" s="14">
-        <v>2.8656929654710845</v>
-      </c>
-      <c r="BL68" s="14">
-        <v>3.5171350932203846E-2</v>
-      </c>
-      <c r="BM68" s="14">
-        <v>8.1069525670619952E-3</v>
-      </c>
-      <c r="BN68" s="14">
-        <v>0.14933907094174137</v>
-      </c>
-      <c r="BO68" s="14">
-        <v>8.1069525670619952E-3</v>
-      </c>
-      <c r="BP68" s="14">
-        <v>0.14933907094174137</v>
-      </c>
+      <c r="AU68" s="17"/>
+      <c r="AV68" s="17"/>
+      <c r="AW68" s="17"/>
+      <c r="AX68" s="17"/>
+      <c r="AY68" s="17"/>
+      <c r="AZ68" s="17"/>
+      <c r="BA68" s="17"/>
+      <c r="BB68" s="17"/>
+      <c r="BC68" s="17"/>
+      <c r="BD68" s="17"/>
+      <c r="BE68" s="17"/>
+      <c r="BF68" s="17"/>
+      <c r="BG68" s="17"/>
+      <c r="BH68" s="17"/>
+      <c r="BI68" s="17"/>
+      <c r="BJ68" s="17"/>
+      <c r="BK68" s="17"/>
+      <c r="BL68" s="17"/>
+      <c r="BM68" s="17"/>
+      <c r="BN68" s="17"/>
+      <c r="BO68" s="17"/>
+      <c r="BP68" s="17"/>
+      <c r="BQ68" s="17"/>
     </row>
-    <row r="69" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>26</v>
       </c>
@@ -39558,8 +39683,31 @@
         <v>1.1131942168706099</v>
       </c>
       <c r="M69" s="8"/>
+      <c r="AU69" s="17"/>
+      <c r="AV69" s="17"/>
+      <c r="AW69" s="17"/>
+      <c r="AX69" s="17"/>
+      <c r="AY69" s="17"/>
+      <c r="AZ69" s="17"/>
+      <c r="BA69" s="17"/>
+      <c r="BB69" s="17"/>
+      <c r="BC69" s="17"/>
+      <c r="BD69" s="17"/>
+      <c r="BE69" s="17"/>
+      <c r="BF69" s="17"/>
+      <c r="BG69" s="17"/>
+      <c r="BH69" s="17"/>
+      <c r="BI69" s="17"/>
+      <c r="BJ69" s="17"/>
+      <c r="BK69" s="17"/>
+      <c r="BL69" s="17"/>
+      <c r="BM69" s="17"/>
+      <c r="BN69" s="17"/>
+      <c r="BO69" s="17"/>
+      <c r="BP69" s="17"/>
+      <c r="BQ69" s="17"/>
     </row>
-    <row r="70" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>25</v>
       </c>
@@ -39596,8 +39744,31 @@
         <v>2.2065870384902602</v>
       </c>
       <c r="M70" s="8"/>
+      <c r="AU70" s="17"/>
+      <c r="AV70" s="17"/>
+      <c r="AW70" s="17"/>
+      <c r="AX70" s="17"/>
+      <c r="AY70" s="17"/>
+      <c r="AZ70" s="17"/>
+      <c r="BA70" s="17"/>
+      <c r="BB70" s="17"/>
+      <c r="BC70" s="17"/>
+      <c r="BD70" s="17"/>
+      <c r="BE70" s="17"/>
+      <c r="BF70" s="17"/>
+      <c r="BG70" s="17"/>
+      <c r="BH70" s="17"/>
+      <c r="BI70" s="17"/>
+      <c r="BJ70" s="17"/>
+      <c r="BK70" s="17"/>
+      <c r="BL70" s="17"/>
+      <c r="BM70" s="17"/>
+      <c r="BN70" s="17"/>
+      <c r="BO70" s="17"/>
+      <c r="BP70" s="17"/>
+      <c r="BQ70" s="17"/>
     </row>
-    <row r="71" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>28</v>
       </c>
@@ -39634,8 +39805,31 @@
         <v>8.4763382350991101</v>
       </c>
       <c r="M71" s="8"/>
+      <c r="AU71" s="17"/>
+      <c r="AV71" s="17"/>
+      <c r="AW71" s="17"/>
+      <c r="AX71" s="17"/>
+      <c r="AY71" s="17"/>
+      <c r="AZ71" s="17"/>
+      <c r="BA71" s="17"/>
+      <c r="BB71" s="17"/>
+      <c r="BC71" s="17"/>
+      <c r="BD71" s="17"/>
+      <c r="BE71" s="17"/>
+      <c r="BF71" s="17"/>
+      <c r="BG71" s="17"/>
+      <c r="BH71" s="17"/>
+      <c r="BI71" s="17"/>
+      <c r="BJ71" s="17"/>
+      <c r="BK71" s="17"/>
+      <c r="BL71" s="17"/>
+      <c r="BM71" s="17"/>
+      <c r="BN71" s="17"/>
+      <c r="BO71" s="17"/>
+      <c r="BP71" s="17"/>
+      <c r="BQ71" s="17"/>
     </row>
-    <row r="72" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>30</v>
       </c>
@@ -39672,8 +39866,31 @@
         <v>9.5412825319663295</v>
       </c>
       <c r="M72" s="8"/>
+      <c r="AU72" s="17"/>
+      <c r="AV72" s="17"/>
+      <c r="AW72" s="17"/>
+      <c r="AX72" s="17"/>
+      <c r="AY72" s="17"/>
+      <c r="AZ72" s="17"/>
+      <c r="BA72" s="17"/>
+      <c r="BB72" s="17"/>
+      <c r="BC72" s="17"/>
+      <c r="BD72" s="17"/>
+      <c r="BE72" s="17"/>
+      <c r="BF72" s="17"/>
+      <c r="BG72" s="17"/>
+      <c r="BH72" s="17"/>
+      <c r="BI72" s="17"/>
+      <c r="BJ72" s="17"/>
+      <c r="BK72" s="17"/>
+      <c r="BL72" s="17"/>
+      <c r="BM72" s="17"/>
+      <c r="BN72" s="17"/>
+      <c r="BO72" s="17"/>
+      <c r="BP72" s="17"/>
+      <c r="BQ72" s="17"/>
     </row>
-    <row r="73" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>32</v>
       </c>
@@ -39710,8 +39927,31 @@
         <v>14.7819327483883</v>
       </c>
       <c r="M73" s="8"/>
+      <c r="AU73" s="17"/>
+      <c r="AV73" s="17"/>
+      <c r="AW73" s="17"/>
+      <c r="AX73" s="17"/>
+      <c r="AY73" s="17"/>
+      <c r="AZ73" s="17"/>
+      <c r="BA73" s="17"/>
+      <c r="BB73" s="17"/>
+      <c r="BC73" s="17"/>
+      <c r="BD73" s="17"/>
+      <c r="BE73" s="17"/>
+      <c r="BF73" s="17"/>
+      <c r="BG73" s="17"/>
+      <c r="BH73" s="17"/>
+      <c r="BI73" s="17"/>
+      <c r="BJ73" s="17"/>
+      <c r="BK73" s="17"/>
+      <c r="BL73" s="17"/>
+      <c r="BM73" s="17"/>
+      <c r="BN73" s="17"/>
+      <c r="BO73" s="17"/>
+      <c r="BP73" s="17"/>
+      <c r="BQ73" s="17"/>
     </row>
-    <row r="74" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>34</v>
       </c>
@@ -39748,6 +39988,29 @@
         <v>48.251680680319097</v>
       </c>
       <c r="M74" s="8"/>
+      <c r="AU74" s="17"/>
+      <c r="AV74" s="17"/>
+      <c r="AW74" s="17"/>
+      <c r="AX74" s="17"/>
+      <c r="AY74" s="17"/>
+      <c r="AZ74" s="17"/>
+      <c r="BA74" s="17"/>
+      <c r="BB74" s="17"/>
+      <c r="BC74" s="17"/>
+      <c r="BD74" s="17"/>
+      <c r="BE74" s="17"/>
+      <c r="BF74" s="17"/>
+      <c r="BG74" s="17"/>
+      <c r="BH74" s="17"/>
+      <c r="BI74" s="17"/>
+      <c r="BJ74" s="17"/>
+      <c r="BK74" s="17"/>
+      <c r="BL74" s="17"/>
+      <c r="BM74" s="17"/>
+      <c r="BN74" s="17"/>
+      <c r="BO74" s="17"/>
+      <c r="BP74" s="17"/>
+      <c r="BQ74" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>